<commit_message>
estimater added, new pipelines
</commit_message>
<xml_diff>
--- a/src/matcher/data/sirketler.xlsx
+++ b/src/matcher/data/sirketler.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aliemre2023/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aliemre2023/Desktop/apache_project/bist100_airflow/src/matcher/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_85E6277334EF7A48278096B52234A9697653D5D5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D724DC44-26E5-E94C-A8C3-DA6C41B3B5B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5091,38 +5091,38 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="34" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="32" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="34" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="35" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5447,7 +5447,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="32" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="6"/>
@@ -5470,7 +5470,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="33" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="6"/>
@@ -6705,7 +6705,7 @@
       </c>
     </row>
     <row r="93" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A93" s="8" t="s">
+      <c r="A93" s="34" t="s">
         <v>224</v>
       </c>
       <c r="B93" s="6"/>
@@ -7506,7 +7506,7 @@
       </c>
     </row>
     <row r="151" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A151" s="9" t="s">
+      <c r="A151" s="35" t="s">
         <v>358</v>
       </c>
       <c r="B151" s="6"/>
@@ -7655,7 +7655,7 @@
       </c>
     </row>
     <row r="162" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A162" s="10" t="s">
+      <c r="A162" s="36" t="s">
         <v>381</v>
       </c>
       <c r="B162" s="6"/>
@@ -7857,7 +7857,7 @@
       </c>
     </row>
     <row r="177" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A177" s="11" t="s">
+      <c r="A177" s="27" t="s">
         <v>415</v>
       </c>
       <c r="B177" s="6"/>
@@ -8479,7 +8479,7 @@
       </c>
     </row>
     <row r="222" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A222" s="12" t="s">
+      <c r="A222" s="28" t="s">
         <v>512</v>
       </c>
       <c r="B222" s="6"/>
@@ -9204,7 +9204,7 @@
       </c>
     </row>
     <row r="275" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A275" s="13" t="s">
+      <c r="A275" s="29" t="s">
         <v>624</v>
       </c>
       <c r="B275" s="6"/>
@@ -9406,7 +9406,7 @@
       </c>
     </row>
     <row r="290" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A290" s="14" t="s">
+      <c r="A290" s="30" t="s">
         <v>655</v>
       </c>
       <c r="B290" s="6"/>
@@ -9857,7 +9857,7 @@
       </c>
     </row>
     <row r="323" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A323" s="15" t="s">
+      <c r="A323" s="31" t="s">
         <v>724</v>
       </c>
       <c r="B323" s="6"/>
@@ -10174,7 +10174,7 @@
       </c>
     </row>
     <row r="346" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A346" s="16" t="s">
+      <c r="A346" s="22" t="s">
         <v>772</v>
       </c>
       <c r="B346" s="6"/>
@@ -10309,7 +10309,7 @@
       </c>
     </row>
     <row r="356" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A356" s="17" t="s">
+      <c r="A356" s="23" t="s">
         <v>792</v>
       </c>
       <c r="B356" s="6"/>
@@ -10710,7 +10710,7 @@
       </c>
     </row>
     <row r="385" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A385" s="18" t="s">
+      <c r="A385" s="24" t="s">
         <v>850</v>
       </c>
       <c r="B385" s="6"/>
@@ -10733,7 +10733,7 @@
       </c>
     </row>
     <row r="387" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A387" s="19" t="s">
+      <c r="A387" s="25" t="s">
         <v>853</v>
       </c>
       <c r="B387" s="6"/>
@@ -11509,7 +11509,7 @@
       </c>
     </row>
     <row r="443" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A443" s="20" t="s">
+      <c r="A443" s="26" t="s">
         <v>970</v>
       </c>
       <c r="B443" s="6"/>
@@ -11672,7 +11672,7 @@
       </c>
     </row>
     <row r="455" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A455" s="21" t="s">
+      <c r="A455" s="17" t="s">
         <v>995</v>
       </c>
       <c r="B455" s="6"/>
@@ -12305,7 +12305,7 @@
       </c>
     </row>
     <row r="501" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A501" s="22" t="s">
+      <c r="A501" s="18" t="s">
         <v>1087</v>
       </c>
       <c r="B501" s="6"/>
@@ -12465,7 +12465,7 @@
       </c>
     </row>
     <row r="513" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A513" s="23" t="s">
+      <c r="A513" s="19" t="s">
         <v>1111</v>
       </c>
       <c r="B513" s="6"/>
@@ -12793,7 +12793,7 @@
       </c>
     </row>
     <row r="537" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A537" s="24" t="s">
+      <c r="A537" s="20" t="s">
         <v>1162</v>
       </c>
       <c r="B537" s="6"/>
@@ -12886,7 +12886,7 @@
       </c>
     </row>
     <row r="544" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A544" s="25" t="s">
+      <c r="A544" s="21" t="s">
         <v>1175</v>
       </c>
       <c r="B544" s="6"/>
@@ -13298,7 +13298,7 @@
       </c>
     </row>
     <row r="574" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A574" s="26" t="s">
+      <c r="A574" s="12" t="s">
         <v>1236</v>
       </c>
       <c r="B574" s="6"/>
@@ -13433,7 +13433,7 @@
       </c>
     </row>
     <row r="584" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A584" s="27" t="s">
+      <c r="A584" s="13" t="s">
         <v>1255</v>
       </c>
       <c r="B584" s="6"/>
@@ -13610,7 +13610,7 @@
       </c>
     </row>
     <row r="597" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A597" s="28" t="s">
+      <c r="A597" s="14" t="s">
         <v>1282</v>
       </c>
       <c r="B597" s="6"/>
@@ -14109,7 +14109,7 @@
       </c>
     </row>
     <row r="633" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A633" s="29" t="s">
+      <c r="A633" s="15" t="s">
         <v>1355</v>
       </c>
       <c r="B633" s="6"/>
@@ -14188,7 +14188,7 @@
       </c>
     </row>
     <row r="639" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A639" s="30" t="s">
+      <c r="A639" s="16" t="s">
         <v>1366</v>
       </c>
       <c r="B639" s="6"/>
@@ -15028,7 +15028,7 @@
       </c>
     </row>
     <row r="700" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A700" s="31" t="s">
+      <c r="A700" s="7" t="s">
         <v>1489</v>
       </c>
       <c r="B700" s="6"/>
@@ -15135,7 +15135,7 @@
       </c>
     </row>
     <row r="708" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A708" s="32" t="s">
+      <c r="A708" s="8" t="s">
         <v>1504</v>
       </c>
       <c r="B708" s="6"/>
@@ -15186,7 +15186,7 @@
       </c>
     </row>
     <row r="712" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A712" s="33" t="s">
+      <c r="A712" s="9" t="s">
         <v>1511</v>
       </c>
       <c r="B712" s="6"/>
@@ -15433,7 +15433,7 @@
       </c>
     </row>
     <row r="730" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A730" s="34" t="s">
+      <c r="A730" s="10" t="s">
         <v>1546</v>
       </c>
       <c r="B730" s="6"/>
@@ -15708,7 +15708,7 @@
       </c>
     </row>
     <row r="750" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A750" s="35" t="s">
+      <c r="A750" s="11" t="s">
         <v>1587</v>
       </c>
       <c r="B750" s="6"/>
@@ -15815,7 +15815,7 @@
       </c>
     </row>
     <row r="758" spans="1:5" ht="19" x14ac:dyDescent="0.25">
-      <c r="A758" s="36" t="s">
+      <c r="A758" s="5" t="s">
         <v>1602</v>
       </c>
       <c r="B758" s="6"/>
@@ -15839,37 +15839,37 @@
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A93:E93"/>
+    <mergeCell ref="A151:E151"/>
+    <mergeCell ref="A162:E162"/>
+    <mergeCell ref="A177:E177"/>
+    <mergeCell ref="A222:E222"/>
+    <mergeCell ref="A275:E275"/>
+    <mergeCell ref="A290:E290"/>
+    <mergeCell ref="A323:E323"/>
+    <mergeCell ref="A346:E346"/>
+    <mergeCell ref="A356:E356"/>
+    <mergeCell ref="A385:E385"/>
+    <mergeCell ref="A387:E387"/>
+    <mergeCell ref="A443:E443"/>
+    <mergeCell ref="A455:E455"/>
+    <mergeCell ref="A501:E501"/>
+    <mergeCell ref="A513:E513"/>
+    <mergeCell ref="A537:E537"/>
+    <mergeCell ref="A544:E544"/>
+    <mergeCell ref="A574:E574"/>
+    <mergeCell ref="A584:E584"/>
+    <mergeCell ref="A597:E597"/>
+    <mergeCell ref="A633:E633"/>
+    <mergeCell ref="A639:E639"/>
     <mergeCell ref="A758:E758"/>
     <mergeCell ref="A700:E700"/>
     <mergeCell ref="A708:E708"/>
     <mergeCell ref="A712:E712"/>
     <mergeCell ref="A730:E730"/>
     <mergeCell ref="A750:E750"/>
-    <mergeCell ref="A574:E574"/>
-    <mergeCell ref="A584:E584"/>
-    <mergeCell ref="A597:E597"/>
-    <mergeCell ref="A633:E633"/>
-    <mergeCell ref="A639:E639"/>
-    <mergeCell ref="A455:E455"/>
-    <mergeCell ref="A501:E501"/>
-    <mergeCell ref="A513:E513"/>
-    <mergeCell ref="A537:E537"/>
-    <mergeCell ref="A544:E544"/>
-    <mergeCell ref="A346:E346"/>
-    <mergeCell ref="A356:E356"/>
-    <mergeCell ref="A385:E385"/>
-    <mergeCell ref="A387:E387"/>
-    <mergeCell ref="A443:E443"/>
-    <mergeCell ref="A177:E177"/>
-    <mergeCell ref="A222:E222"/>
-    <mergeCell ref="A275:E275"/>
-    <mergeCell ref="A290:E290"/>
-    <mergeCell ref="A323:E323"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A93:E93"/>
-    <mergeCell ref="A151:E151"/>
-    <mergeCell ref="A162:E162"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>